<commit_message>
Update workbook poster data
</commit_message>
<xml_diff>
--- a/MCU.xlsx
+++ b/MCU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419CDABF-3F34-4F9F-9FE7-A9830B61CE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49619F47-FC6F-48D5-8A52-B08DDCE979AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MCUDATASHEET!$A$1:$T$1062</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -12221,6 +12234,7 @@
     <col min="9" max="9" width="23.85546875" style="3" customWidth="1"/>
     <col min="10" max="10" width="19.85546875" style="3" customWidth="1"/>
     <col min="13" max="13" width="30.85546875" customWidth="1"/>
+    <col min="18" max="18" width="45.42578125" customWidth="1"/>
     <col min="19" max="19" width="56.42578125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>